<commit_message>
Incorpora la matriz de Control de Inventarios al consolidado
La matriz GE-SO-CI-D1 cubre los puestos Tecnico de Inventario (3 personas) y
Analista de Inventario (1), ambos con denominacion coincidente con el head
count, sin necesidad de equivalencias.

Operaciones pasa de 14 a 16 cargos analizados (72%). El total sube a 52 de 70
cargos (74%) y 76 de 101 personas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSq5v2aoJeLSvtorf4qgpi
</commit_message>
<xml_diff>
--- a/Cobertura_IPERC_Administrativos_CAR.xlsx
+++ b/Cobertura_IPERC_Administrativos_CAR.xlsx
@@ -18,9 +18,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1. Alcance y criterios'!$A$4:$C$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Resumen por área'!$A$4:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Matriz consolidada'!$A$4:$J$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5. Observaciones'!$A$4:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -855,22 +855,22 @@
         <v>22</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>37</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
@@ -1086,22 +1086,22 @@
         <v>70</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>101</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I13" s="14" t="inlineStr"/>
     </row>
@@ -2922,21 +2922,25 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F44" s="17" t="inlineStr">
-        <is>
-          <t>SIN ANALIZAR</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr"/>
-      <c r="H44" s="5" t="inlineStr"/>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>ANALIZADO</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>GE-SO-CI-D1</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Analista de Inventario</t>
+        </is>
+      </c>
       <c r="I44" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="5" t="inlineStr">
-        <is>
-          <t>Requiere elaboración de matriz IPERC</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="J44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3786,21 +3790,25 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F64" s="17" t="inlineStr">
-        <is>
-          <t>SIN ANALIZAR</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr"/>
-      <c r="H64" s="5" t="inlineStr"/>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>ANALIZADO</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>GE-SO-CI-D1</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Técnico de Inventario</t>
+        </is>
+      </c>
       <c r="I64" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" s="5" t="inlineStr">
-        <is>
-          <t>Requiere elaboración de matriz IPERC</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="J64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4258,7 +4266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4373,20 +4381,20 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>QSE &amp; Operational Excellence</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>TECNICO DE INVENTARIO</t>
+          <t>COORDINADOR DE EXCELENCIA OPERACIONAL</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BC Adm</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -4396,7 +4404,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>4950 INVENTARY</t>
+          <t>4650 EXCELENCIA OPERACIONAL</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -4410,30 +4418,30 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>QSE &amp; Operational Excellence</t>
+          <t>Gerencia</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>COORDINADOR DE EXCELENCIA OPERACIONAL</t>
+          <t>CHOFER</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>BC Adm</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Quevedo</t>
+          <t>Samborondon</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>4650 EXCELENCIA OPERACIONAL</t>
+          <t>5800 GENERAL MANAGEMENT</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -4452,7 +4460,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>CHOFER</t>
+          <t>GERENTE GENERAL</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
@@ -4460,12 +4468,12 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>BC Adm</t>
+          <t>Top Management</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Samborondon</t>
+          <t>Quevedo</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -4484,12 +4492,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Gerencia</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>GERENTE GENERAL</t>
+          <t>JUNIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
@@ -4497,17 +4505,17 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Top Management</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Quevedo</t>
+          <t>Samborondon</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>5800 GENERAL MANAGEMENT</t>
+          <t>5930 3ACM Expenses</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -4521,12 +4529,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>IT&amp;FIN</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>JUNIOR BUSINESS CONTROLLER</t>
+          <t>ANALISTA DE IMPUESTOS</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
@@ -4544,7 +4552,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>5930 3ACM Expenses</t>
+          <t>5300 FINANCE</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -4563,7 +4571,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>ANALISTA DE IMPUESTOS</t>
+          <t>ANALISTA DE REDES</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -4581,7 +4589,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>5300 FINANCE</t>
+          <t>5400 IT</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -4600,7 +4608,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>ANALISTA DE REDES</t>
+          <t>DIRECTOR FINANCIERO</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
@@ -4608,7 +4616,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Top Management</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -4618,7 +4626,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>5400 IT</t>
+          <t>5300 FINANCE</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -4637,7 +4645,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>DIRECTOR FINANCIERO</t>
+          <t>GERENTE FINANCIERO</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -4645,7 +4653,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Top Management</t>
+          <t>Middle Management</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -4674,7 +4682,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>GERENTE FINANCIERO</t>
+          <t>JEFE  DE DESARROLLO DE APLICACIONES</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
@@ -4682,7 +4690,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Middle Management</t>
+          <t>Low Management</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -4692,7 +4700,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>5300 FINANCE</t>
+          <t>5400 IT</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -4711,7 +4719,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>JEFE  DE DESARROLLO DE APLICACIONES</t>
+          <t>JUNIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -4719,7 +4727,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Low Management</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -4729,7 +4737,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>5400 IT</t>
+          <t>5934 BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -4748,7 +4756,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>JUNIOR BUSINESS CONTROLLER</t>
+          <t>MENSAJERO / REPARTIDOR</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
@@ -4756,7 +4764,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>BC Adm</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -4766,7 +4774,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>5934 BUSINESS CONTROLLER</t>
+          <t>5300 FINANCE</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -4785,7 +4793,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>MENSAJERO / REPARTIDOR</t>
+          <t>SENIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
@@ -4793,7 +4801,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>BC Adm</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -4803,7 +4811,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>5300 FINANCE</t>
+          <t>5934 BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -4817,12 +4825,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>IT&amp;FIN</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>SENIOR BUSINESS CONTROLLER</t>
+          <t>APRENDIZ</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
@@ -4830,17 +4838,17 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>BC Adm</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Samborondon</t>
+          <t>Quevedo</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>5934 BUSINESS CONTROLLER</t>
+          <t>3801 PLANTABAL MANTENANCE #1</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -4859,7 +4867,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>ANALISTA DE INVENTARIO</t>
+          <t>DIRECTOR DE OPERACIONES</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
@@ -4867,7 +4875,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Top Management</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -4877,7 +4885,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>4950 INVENTARY</t>
+          <t>4800 PLANTABAL OPERATIONS MNG STAFF</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -4896,7 +4904,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>APRENDIZ</t>
+          <t>GERENTE DE PRODUCCION</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
@@ -4904,7 +4912,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>BC Adm</t>
+          <t>Middle Management</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -4914,7 +4922,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>3801 PLANTABAL MANTENANCE #1</t>
+          <t>4800 PLANTABAL OPERATIONS MNG STAFF</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -4933,7 +4941,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>DIRECTOR DE OPERACIONES</t>
+          <t>JEFE DE BODEGA</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
@@ -4941,7 +4949,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Top Management</t>
+          <t>Low Management</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -4951,7 +4959,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>4800 PLANTABAL OPERATIONS MNG STAFF</t>
+          <t>2500 SERVICE CENTER</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -4970,7 +4978,7 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>GERENTE DE PRODUCCION</t>
+          <t>JEFE DE PRODUCCION</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
@@ -4978,7 +4986,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Middle Management</t>
+          <t>Low Management</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -4999,82 +5007,8 @@
       <c r="H22" s="5" t="inlineStr"/>
       <c r="I22" s="5" t="inlineStr"/>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>JEFE DE BODEGA</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Low Management</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Quevedo</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>2500 SERVICE CENTER</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Elaborar matriz IPERC para el puesto</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>JEFE DE PRODUCCION</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Low Management</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Quevedo</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>4800 PLANTABAL OPERATIONS MNG STAFF</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>Elaborar matriz IPERC para el puesto</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr"/>
-      <c r="I24" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:I24"/>
+  <autoFilter ref="A4:I22"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -5608,7 +5542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5752,329 +5686,357 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-EHS-D1</t>
+          <t>GE-SO-CI-D1</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>EHS</t>
+          <t>Técnico de Inventario</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Ingeniero de seguridad y ambiente (13) · Tecnico de seguridad y ambiente (16)</t>
+          <t>Técnico de Inventario (14) · Analista de Inventario (10)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>a5c35af4-GE-SO-EHS-D1-_EHS.xlsx</t>
+          <t>7d905433-GE-SO-CI-D1_-_Control_de_Inventarios.xlsx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-FI-D1</t>
+          <t>GE-SO-EHS-D1</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Finanzas</t>
+          <t>EHS</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Coordinador Contable y de Impuestos (7) · Analista financiero (4) · Coordinador Contable (8) · Jefe de Contabilidad e Impuestos (9) · Coordinador de Tesoreria (6)</t>
+          <t>Ingeniero de seguridad y ambiente (13) · Tecnico de seguridad y ambiente (16)</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>109ebe9e-GE-SO-FI-D1_-_Finanzas.xlsx</t>
+          <t>a5c35af4-GE-SO-EHS-D1-_EHS.xlsx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-IT-D1</t>
+          <t>GE-SO-FI-D1</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Help Desk</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Help Desk (10) · Desarrollador JR (6) · Gerente tecnologico (6) · Analista de desarrollo y sistema (5)</t>
+          <t>Coordinador Contable y de Impuestos (7) · Analista financiero (4) · Coordinador Contable (8) · Jefe de Contabilidad e Impuestos (9) · Coordinador de Tesoreria (6)</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>7794a690-GE-SO-IT-D1_-_IT.xlsx</t>
+          <t>109ebe9e-GE-SO-FI-D1_-_Finanzas.xlsx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-LE-D1</t>
+          <t>GE-SO-IT-D1</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Help Desk</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Asistente Legal (11) · Analista Legal (10) · Coordinador/a de Asuntos Legales (10)</t>
+          <t>Help Desk (10) · Desarrollador JR (6) · Gerente tecnologico (6) · Analista de desarrollo y sistema (5)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>904e5c44-GE-SO-LE-D1_-_Legal.xlsx</t>
+          <t>7794a690-GE-SO-IT-D1_-_IT.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-MA-D1</t>
+          <t>GE-SO-LE-D1</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Mantenimiento - Administrativos</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>156</v>
+        <v>31</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Gerente JR de mantenimiento (20) · Jefe de mantenimiento (42) · Planificador de mantenimiento (21) · Supervisor de mantenimiento (38) · Auxiliar administrativo (35)</t>
+          <t>Asistente Legal (11) · Analista Legal (10) · Coordinador/a de Asuntos Legales (10)</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>271a4bea-GE-SO-MA-D1_-_Mantenimiento.xlsx</t>
+          <t>904e5c44-GE-SO-LE-D1_-_Legal.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-PGS-D1</t>
+          <t>GE-SO-MA-D1</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Engicore</t>
+          <t>Mantenimiento - Administrativos</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>32</v>
+        <v>156</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Jefe de Diseño e Ingenieria (9) · Ingeniero de Diseño e Ingenieria (14) · Analista de Diseño e Ingenieria (9)</t>
+          <t>Gerente JR de mantenimiento (20) · Jefe de mantenimiento (42) · Planificador de mantenimiento (21) · Supervisor de mantenimiento (38) · Auxiliar administrativo (35)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>f4a8175b-GE-SO-PGS-D1_-_Engicore.xlsx</t>
+          <t>271a4bea-GE-SO-MA-D1_-_Mantenimiento.xlsx</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-PO-D1</t>
+          <t>GE-SO-PGS-D1</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Planificación y Logística</t>
+          <t>Engicore</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Jefe de Planificación y Logística (11) · Coordinador de Supply Chain (6) · Programador de Producción (8) · Analista de Supply Chain (6)</t>
+          <t>Jefe de Diseño e Ingenieria (9) · Ingeniero de Diseño e Ingenieria (14) · Analista de Diseño e Ingenieria (9)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>1fa9982d-GE-SO-PO-D1_-_Planificaci_n_y_Log_stica.xlsx</t>
+          <t>f4a8175b-GE-SO-PGS-D1_-_Engicore.xlsx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-PY-D1</t>
+          <t>GE-SO-PO-D1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Proyectos</t>
+          <t>Planificación y Logística</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Jefe de Proyectos (20) · Ingeniero de Proyectos (15) · Analista de Proyectos (16)</t>
+          <t>Jefe de Planificación y Logística (11) · Coordinador de Supply Chain (6) · Programador de Producción (8) · Analista de Supply Chain (6)</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>933cde5a-GE-SO-PY-D1_-_Proyectos.xlsx</t>
+          <t>1fa9982d-GE-SO-PO-D1_-_Planificaci_n_y_Log_stica.xlsx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-SC-D1</t>
+          <t>GE-SO-PY-D1</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Proyectos</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
         <v>3</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Analista Supply Chain (13) · Analista Compras (14) · Jefe de Compras (13)</t>
+          <t>Jefe de Proyectos (20) · Ingeniero de Proyectos (15) · Analista de Proyectos (16)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>9c752964-GE-SO-SC-D1_-_Compras.xlsx</t>
+          <t>933cde5a-GE-SO-PY-D1_-_Proyectos.xlsx</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-SF-D1</t>
+          <t>GE-SO-SC-D1</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Salud Ocupacional</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Medico Ocupacional (18) · Enfermero Ocupacional (10) · Auxiliar de servicios de salud (11)</t>
+          <t>Analista Supply Chain (13) · Analista Compras (14) · Jefe de Compras (13)</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>cf092d8f-GE-SO-SF-D1_-_Salud_ocupacional.xlsx</t>
+          <t>9c752964-GE-SO-SC-D1_-_Compras.xlsx</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-TH-D1</t>
+          <t>GE-SO-SF-D1</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>RECURSOS HUMANOS</t>
+          <t>Salud Ocupacional</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>339</v>
+        <v>39</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>HR DIRECTOR AMERICAS (36) · HR BUSINNES PARTNER AMERICAS (42) · BUSINNES PARTNER DE RECURSOS HUMANOS (28) · COORDINADORA DE DESARROLLO ORGANIZACIONAL (49) · PEOPLE OPERATIONS PARTNER (42) · ANALISTA DE RECURSOS HUMANOS (72) · ANALISTA DE RECURSOS HUMANOS Y NÓMINA (28) · ANALISTA DE DESARROLLO ORGANIZACIONAL (42)</t>
+          <t>Medico Ocupacional (18) · Enfermero Ocupacional (10) · Auxiliar de servicios de salud (11)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>b206b7b5-GE-SO-TH-D1_-_RRHH.xlsx</t>
+          <t>cf092d8f-GE-SO-SF-D1_-_Salud_ocupacional.xlsx</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>GE-SO-TH-D1</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>RECURSOS HUMANOS</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>339</v>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>HR DIRECTOR AMERICAS (36) · HR BUSINNES PARTNER AMERICAS (42) · BUSINNES PARTNER DE RECURSOS HUMANOS (28) · COORDINADORA DE DESARROLLO ORGANIZACIONAL (49) · PEOPLE OPERATIONS PARTNER (42) · ANALISTA DE RECURSOS HUMANOS (72) · ANALISTA DE RECURSOS HUMANOS Y NÓMINA (28) · ANALISTA DE DESARROLLO ORGANIZACIONAL (42)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>b206b7b5-GE-SO-TH-D1_-_RRHH.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>1083</v>
-      </c>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>1107</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F19"/>
+  <autoFilter ref="A4:F20"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Incorpora las matrices de Excelencia Operacional y Operations Mng Staff
GE-SO-EO-D1 cubre el Coordinador de Excelencia Operacional (2 personas), con lo
que QSE & Operational Excellence queda conforme: cuarta area al 100%.

GE-SO-RL-D35 cubre Director de Operaciones y Gerente de Produccion, y eleva
Operaciones al 82%. Su codigo sigue otro patron de numeracion (RL-D35) que el
extractor reconoce sin cambios.

El total pasa a 55 de 70 cargos (79%) y 80 de 101 personas. Quedan 15 brechas,
la mas pesada Supervisor de Produccion con 7 personas.

Queda pendiente de validacion la denominacion 'Jefe de Produccion (MV y Secado)'
de GE-SO-RL-D35, que el control reporta como puesto sin clasificar por no
coincidir con 'JEFE DE PRODUCCION' del head count.

Agrega .gitignore para los artefactos de Python.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSq5v2aoJeLSvtorf4qgpi
</commit_message>
<xml_diff>
--- a/Cobertura_IPERC_Administrativos_CAR.xlsx
+++ b/Cobertura_IPERC_Administrativos_CAR.xlsx
@@ -18,9 +18,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1. Alcance y criterios'!$A$4:$C$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Resumen por área'!$A$4:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Matriz consolidada'!$A$4:$J$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$I$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5. Observaciones'!$A$4:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5. Observaciones'!$A$4:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -163,10 +163,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -564,7 +564,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 29/09/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 29/09/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -855,22 +855,22 @@
         <v>22</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>37</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
@@ -947,47 +947,47 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>QSE &amp; Operational Excellence</t>
+          <t>ADM-L&amp;RH</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>CON BRECHAS</t>
+        <v>0</v>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>CONFORME</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>ADM-L&amp;RH</t>
+          <t>ESG/Lab</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>0</v>
@@ -996,15 +996,15 @@
         <v>100</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H10" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="12" t="inlineStr">
+      <c r="I10" s="13" t="inlineStr">
         <is>
           <t>CONFORME</t>
         </is>
@@ -1013,14 +1013,14 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>ESG/Lab</t>
+          <t>Engicore</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -1029,15 +1029,15 @@
         <v>100</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>CONFORME</t>
         </is>
@@ -1046,14 +1046,14 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Engicore</t>
+          <t>QSE &amp; Operational Excellence</t>
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>0</v>
@@ -1062,15 +1062,15 @@
         <v>100</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="12" t="inlineStr">
+      <c r="I12" s="13" t="inlineStr">
         <is>
           <t>CONFORME</t>
         </is>
@@ -1086,22 +1086,22 @@
         <v>70</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>101</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I13" s="14" t="inlineStr"/>
     </row>
@@ -1146,7 +1146,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 29/09/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1270,7 +1270,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1314,7 +1314,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1358,7 +1358,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1402,7 +1402,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1446,23 +1446,23 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-MA-D1 / GE-SO-SF-D1</t>
+          <t>GE-SO-MA-D1 / GE-SO-RL-D35 / GE-SO-SF-D1</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo / Auxiliar de servicios de salud</t>
+          <t>Auxiliar Administrativo / Auxiliar administrativo / Auxiliar de servicios de salud</t>
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
@@ -1494,7 +1494,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1538,7 +1538,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1582,7 +1582,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1626,7 +1626,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1674,7 +1674,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1718,7 +1718,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1762,7 +1762,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1806,7 +1806,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1850,7 +1850,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F19" s="13" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1894,7 +1894,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F20" s="12" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1938,7 +1938,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -1982,7 +1982,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F22" s="12" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2026,7 +2026,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2074,7 +2074,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2318,7 +2318,7 @@
           <t>Samborondon</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2362,7 +2362,7 @@
           <t>Samborondon</t>
         </is>
       </c>
-      <c r="F31" s="13" t="inlineStr">
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2410,7 +2410,7 @@
           <t>Samborondon</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
+      <c r="F32" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2454,7 +2454,7 @@
           <t>Samborondon</t>
         </is>
       </c>
-      <c r="F33" s="13" t="inlineStr">
+      <c r="F33" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2498,7 +2498,7 @@
           <t>Samborondon</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr">
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2622,7 +2622,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F37" s="13" t="inlineStr">
+      <c r="F37" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2786,7 +2786,7 @@
           <t>Samborondon</t>
         </is>
       </c>
-      <c r="F41" s="13" t="inlineStr">
+      <c r="F41" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2874,7 +2874,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F43" s="13" t="inlineStr">
+      <c r="F43" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2922,7 +2922,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F44" s="12" t="inlineStr">
+      <c r="F44" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -2966,7 +2966,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F45" s="13" t="inlineStr">
+      <c r="F45" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3010,7 +3010,7 @@
           <t>Quevedo / Samborondon</t>
         </is>
       </c>
-      <c r="F46" s="12" t="inlineStr">
+      <c r="F46" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3098,23 +3098,23 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F48" s="12" t="inlineStr">
+      <c r="F48" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-MA-D1 / GE-SO-SF-D1</t>
+          <t>GE-SO-MA-D1 / GE-SO-RL-D35 / GE-SO-SF-D1</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo / Auxiliar de servicios de salud</t>
+          <t>Auxiliar Administrativo / Auxiliar administrativo / Auxiliar de servicios de salud</t>
         </is>
       </c>
       <c r="I48" s="9" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
@@ -3146,7 +3146,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F49" s="13" t="inlineStr">
+      <c r="F49" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3190,21 +3190,25 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F50" s="17" t="inlineStr">
-        <is>
-          <t>SIN ANALIZAR</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr"/>
-      <c r="H50" s="5" t="inlineStr"/>
+      <c r="F50" s="13" t="inlineStr">
+        <is>
+          <t>ANALIZADO</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>GE-SO-RL-D35</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>Director de Operaciones</t>
+        </is>
+      </c>
       <c r="I50" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" s="5" t="inlineStr">
-        <is>
-          <t>Requiere elaboración de matriz IPERC</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="J50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3230,21 +3234,25 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F51" s="17" t="inlineStr">
-        <is>
-          <t>SIN ANALIZAR</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr"/>
-      <c r="H51" s="4" t="inlineStr"/>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>ANALIZADO</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>GE-SO-RL-D35</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Gerente de Producción</t>
+        </is>
+      </c>
       <c r="I51" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>Requiere elaboración de matriz IPERC</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -3270,7 +3278,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F52" s="12" t="inlineStr">
+      <c r="F52" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3314,7 +3322,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F53" s="13" t="inlineStr">
+      <c r="F53" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3398,7 +3406,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F55" s="13" t="inlineStr">
+      <c r="F55" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3446,7 +3454,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F56" s="12" t="inlineStr">
+      <c r="F56" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3490,7 +3498,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F57" s="13" t="inlineStr">
+      <c r="F57" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3574,7 +3582,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F59" s="13" t="inlineStr">
+      <c r="F59" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3618,7 +3626,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F60" s="12" t="inlineStr">
+      <c r="F60" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3662,7 +3670,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F61" s="13" t="inlineStr">
+      <c r="F61" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3706,7 +3714,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F62" s="12" t="inlineStr">
+      <c r="F62" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3790,7 +3798,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F64" s="12" t="inlineStr">
+      <c r="F64" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3834,7 +3842,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F65" s="13" t="inlineStr">
+      <c r="F65" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3878,7 +3886,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F66" s="12" t="inlineStr">
+      <c r="F66" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -3922,21 +3930,25 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F67" s="17" t="inlineStr">
-        <is>
-          <t>SIN ANALIZAR</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr"/>
-      <c r="H67" s="4" t="inlineStr"/>
+      <c r="F67" s="12" t="inlineStr">
+        <is>
+          <t>ANALIZADO</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>GE-SO-EO-D1</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>Coordinador de Excelencia Operacional</t>
+        </is>
+      </c>
       <c r="I67" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>Requiere elaboración de matriz IPERC</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="J67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -3962,7 +3974,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F68" s="12" t="inlineStr">
+      <c r="F68" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -4006,7 +4018,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F69" s="13" t="inlineStr">
+      <c r="F69" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -4050,7 +4062,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F70" s="12" t="inlineStr">
+      <c r="F70" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -4098,7 +4110,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F71" s="13" t="inlineStr">
+      <c r="F71" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -4142,7 +4154,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F72" s="12" t="inlineStr">
+      <c r="F72" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -4186,7 +4198,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F73" s="13" t="inlineStr">
+      <c r="F73" s="12" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -4230,7 +4242,7 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F74" s="12" t="inlineStr">
+      <c r="F74" s="13" t="inlineStr">
         <is>
           <t>ANALIZADO</t>
         </is>
@@ -4266,7 +4278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4290,7 +4302,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 29/09/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -4381,30 +4393,30 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>QSE &amp; Operational Excellence</t>
+          <t>Gerencia</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>COORDINADOR DE EXCELENCIA OPERACIONAL</t>
+          <t>CHOFER</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>BC Adm</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Quevedo</t>
+          <t>Samborondon</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>4650 EXCELENCIA OPERACIONAL</t>
+          <t>5800 GENERAL MANAGEMENT</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -4423,7 +4435,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>CHOFER</t>
+          <t>GERENTE GENERAL</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -4431,12 +4443,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>BC Adm</t>
+          <t>Top Management</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Samborondon</t>
+          <t>Quevedo</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -4455,12 +4467,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Gerencia</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>GERENTE GENERAL</t>
+          <t>JUNIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
@@ -4468,17 +4480,17 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Top Management</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Quevedo</t>
+          <t>Samborondon</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>5800 GENERAL MANAGEMENT</t>
+          <t>5930 3ACM Expenses</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -4492,12 +4504,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>IT&amp;FIN</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>JUNIOR BUSINESS CONTROLLER</t>
+          <t>ANALISTA DE IMPUESTOS</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
@@ -4515,7 +4527,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>5930 3ACM Expenses</t>
+          <t>5300 FINANCE</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -4534,7 +4546,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>ANALISTA DE IMPUESTOS</t>
+          <t>ANALISTA DE REDES</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
@@ -4552,7 +4564,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>5300 FINANCE</t>
+          <t>5400 IT</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -4571,7 +4583,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>ANALISTA DE REDES</t>
+          <t>DIRECTOR FINANCIERO</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -4579,7 +4591,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>Top Management</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -4589,7 +4601,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>5400 IT</t>
+          <t>5300 FINANCE</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -4608,7 +4620,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>DIRECTOR FINANCIERO</t>
+          <t>GERENTE FINANCIERO</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
@@ -4616,7 +4628,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Top Management</t>
+          <t>Middle Management</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -4645,7 +4657,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>GERENTE FINANCIERO</t>
+          <t>JEFE  DE DESARROLLO DE APLICACIONES</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -4653,7 +4665,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Middle Management</t>
+          <t>Low Management</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -4663,7 +4675,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>5300 FINANCE</t>
+          <t>5400 IT</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -4682,7 +4694,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>JEFE  DE DESARROLLO DE APLICACIONES</t>
+          <t>JUNIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
@@ -4690,7 +4702,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Low Management</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -4700,7 +4712,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>5400 IT</t>
+          <t>5934 BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -4719,7 +4731,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>JUNIOR BUSINESS CONTROLLER</t>
+          <t>MENSAJERO / REPARTIDOR</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -4727,7 +4739,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>BC Adm</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -4737,7 +4749,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>5934 BUSINESS CONTROLLER</t>
+          <t>5300 FINANCE</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -4756,7 +4768,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>MENSAJERO / REPARTIDOR</t>
+          <t>SENIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
@@ -4764,7 +4776,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>BC Adm</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -4774,7 +4786,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>5300 FINANCE</t>
+          <t>5934 BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -4788,12 +4800,12 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>IT&amp;FIN</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>SENIOR BUSINESS CONTROLLER</t>
+          <t>APRENDIZ</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
@@ -4801,17 +4813,17 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>BC Adm</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Samborondon</t>
+          <t>Quevedo</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>5934 BUSINESS CONTROLLER</t>
+          <t>3801 PLANTABAL MANTENANCE #1</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -4830,7 +4842,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>APRENDIZ</t>
+          <t>JEFE DE BODEGA</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
@@ -4838,7 +4850,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>BC Adm</t>
+          <t>Low Management</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -4848,7 +4860,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>3801 PLANTABAL MANTENANCE #1</t>
+          <t>2500 SERVICE CENTER</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -4867,7 +4879,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>DIRECTOR DE OPERACIONES</t>
+          <t>JEFE DE PRODUCCION</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
@@ -4875,7 +4887,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Top Management</t>
+          <t>Low Management</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -4896,119 +4908,8 @@
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr"/>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>GERENTE DE PRODUCCION</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Middle Management</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Quevedo</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>4800 PLANTABAL OPERATIONS MNG STAFF</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Elaborar matriz IPERC para el puesto</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>JEFE DE BODEGA</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Low Management</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Quevedo</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>2500 SERVICE CENTER</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Elaborar matriz IPERC para el puesto</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>JEFE DE PRODUCCION</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Low Management</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Quevedo</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>4800 PLANTABAL OPERATIONS MNG STAFF</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>Elaborar matriz IPERC para el puesto</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr"/>
-      <c r="I22" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:I22"/>
+  <autoFilter ref="A4:I19"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -5023,7 +4924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5045,7 +4946,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 29/09/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -5526,8 +5427,41 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>GE-SO-RL-D35</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Jefe de Producción (MV y Secado)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>(no consta)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>SIN CLASIFICAR - detectado este mes</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Puesto evaluado en la matriz que no aparece en el head count del mes</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Definir si es cargo nuevo, denominación alterna o cargo suprimido</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G16"/>
+  <autoFilter ref="A4:G17"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -5542,7 +5476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5563,7 +5497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 29/09/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -5742,301 +5676,357 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-FI-D1</t>
+          <t>GE-SO-EO-D1</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Finanzas</t>
+          <t>Excelencia Operacional</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Coordinador Contable y de Impuestos (7) · Analista financiero (4) · Coordinador Contable (8) · Jefe de Contabilidad e Impuestos (9) · Coordinador de Tesoreria (6)</t>
+          <t>Coordinador de Excelencia Operacional (12)</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>109ebe9e-GE-SO-FI-D1_-_Finanzas.xlsx</t>
+          <t>6e2db6dc-GE-SO-EO-D1_-_Excelencia_Operacional.xlsx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-IT-D1</t>
+          <t>GE-SO-FI-D1</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Help Desk</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Help Desk (10) · Desarrollador JR (6) · Gerente tecnologico (6) · Analista de desarrollo y sistema (5)</t>
+          <t>Coordinador Contable y de Impuestos (7) · Analista financiero (4) · Coordinador Contable (8) · Jefe de Contabilidad e Impuestos (9) · Coordinador de Tesoreria (6)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>7794a690-GE-SO-IT-D1_-_IT.xlsx</t>
+          <t>109ebe9e-GE-SO-FI-D1_-_Finanzas.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-LE-D1</t>
+          <t>GE-SO-IT-D1</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Help Desk</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Asistente Legal (11) · Analista Legal (10) · Coordinador/a de Asuntos Legales (10)</t>
+          <t>Help Desk (10) · Desarrollador JR (6) · Gerente tecnologico (6) · Analista de desarrollo y sistema (5)</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>904e5c44-GE-SO-LE-D1_-_Legal.xlsx</t>
+          <t>7794a690-GE-SO-IT-D1_-_IT.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-MA-D1</t>
+          <t>GE-SO-LE-D1</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Mantenimiento - Administrativos</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>156</v>
+        <v>31</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Gerente JR de mantenimiento (20) · Jefe de mantenimiento (42) · Planificador de mantenimiento (21) · Supervisor de mantenimiento (38) · Auxiliar administrativo (35)</t>
+          <t>Asistente Legal (11) · Analista Legal (10) · Coordinador/a de Asuntos Legales (10)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>271a4bea-GE-SO-MA-D1_-_Mantenimiento.xlsx</t>
+          <t>904e5c44-GE-SO-LE-D1_-_Legal.xlsx</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-PGS-D1</t>
+          <t>GE-SO-MA-D1</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Engicore</t>
+          <t>Mantenimiento - Administrativos</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>32</v>
+        <v>156</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Jefe de Diseño e Ingenieria (9) · Ingeniero de Diseño e Ingenieria (14) · Analista de Diseño e Ingenieria (9)</t>
+          <t>Gerente JR de mantenimiento (20) · Jefe de mantenimiento (42) · Planificador de mantenimiento (21) · Supervisor de mantenimiento (38) · Auxiliar administrativo (35)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>f4a8175b-GE-SO-PGS-D1_-_Engicore.xlsx</t>
+          <t>271a4bea-GE-SO-MA-D1_-_Mantenimiento.xlsx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-PO-D1</t>
+          <t>GE-SO-PGS-D1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Planificación y Logística</t>
+          <t>Engicore</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Jefe de Planificación y Logística (11) · Coordinador de Supply Chain (6) · Programador de Producción (8) · Analista de Supply Chain (6)</t>
+          <t>Jefe de Diseño e Ingenieria (9) · Ingeniero de Diseño e Ingenieria (14) · Analista de Diseño e Ingenieria (9)</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1fa9982d-GE-SO-PO-D1_-_Planificaci_n_y_Log_stica.xlsx</t>
+          <t>f4a8175b-GE-SO-PGS-D1_-_Engicore.xlsx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-PY-D1</t>
+          <t>GE-SO-PO-D1</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Proyectos</t>
+          <t>Planificación y Logística</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Jefe de Proyectos (20) · Ingeniero de Proyectos (15) · Analista de Proyectos (16)</t>
+          <t>Jefe de Planificación y Logística (11) · Coordinador de Supply Chain (6) · Programador de Producción (8) · Analista de Supply Chain (6)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>933cde5a-GE-SO-PY-D1_-_Proyectos.xlsx</t>
+          <t>1fa9982d-GE-SO-PO-D1_-_Planificaci_n_y_Log_stica.xlsx</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-SC-D1</t>
+          <t>GE-SO-PY-D1</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Proyectos</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Analista Supply Chain (13) · Analista Compras (14) · Jefe de Compras (13)</t>
+          <t>Jefe de Proyectos (20) · Ingeniero de Proyectos (15) · Analista de Proyectos (16)</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>9c752964-GE-SO-SC-D1_-_Compras.xlsx</t>
+          <t>933cde5a-GE-SO-PY-D1_-_Proyectos.xlsx</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-SF-D1</t>
+          <t>GE-SO-RL-D35</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Salud Ocupacional</t>
+          <t>Operations Mng Staff</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Medico Ocupacional (18) · Enfermero Ocupacional (10) · Auxiliar de servicios de salud (11)</t>
+          <t>Director de Operaciones (14) · Gerente de Producción (16) · Jefe de Producción (MV y Secado) (18) · Auxiliar Administrativo (12)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>cf092d8f-GE-SO-SF-D1_-_Salud_ocupacional.xlsx</t>
+          <t>fe6c6893-Matriz_IPERC_Plantabal_Operations_Mng_Staff.xlsx</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-TH-D1</t>
+          <t>GE-SO-SC-D1</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>RECURSOS HUMANOS</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>339</v>
+        <v>40</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>HR DIRECTOR AMERICAS (36) · HR BUSINNES PARTNER AMERICAS (42) · BUSINNES PARTNER DE RECURSOS HUMANOS (28) · COORDINADORA DE DESARROLLO ORGANIZACIONAL (49) · PEOPLE OPERATIONS PARTNER (42) · ANALISTA DE RECURSOS HUMANOS (72) · ANALISTA DE RECURSOS HUMANOS Y NÓMINA (28) · ANALISTA DE DESARROLLO ORGANIZACIONAL (42)</t>
+          <t>Analista Supply Chain (13) · Analista Compras (14) · Jefe de Compras (13)</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>b206b7b5-GE-SO-TH-D1_-_RRHH.xlsx</t>
+          <t>9c752964-GE-SO-SC-D1_-_Compras.xlsx</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>GE-SO-SF-D1</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Salud Ocupacional</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Medico Ocupacional (18) · Enfermero Ocupacional (10) · Auxiliar de servicios de salud (11)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>cf092d8f-GE-SO-SF-D1_-_Salud_ocupacional.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>GE-SO-TH-D1</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>RECURSOS HUMANOS</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>339</v>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>HR DIRECTOR AMERICAS (36) · HR BUSINNES PARTNER AMERICAS (42) · BUSINNES PARTNER DE RECURSOS HUMANOS (28) · COORDINADORA DE DESARROLLO ORGANIZACIONAL (49) · PEOPLE OPERATIONS PARTNER (42) · ANALISTA DE RECURSOS HUMANOS (72) · ANALISTA DE RECURSOS HUMANOS Y NÓMINA (28) · ANALISTA DE DESARROLLO ORGANIZACIONAL (42)</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>b206b7b5-GE-SO-TH-D1_-_RRHH.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="9" t="n">
-        <v>54</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>1107</v>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>1179</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F20"/>
+  <autoFilter ref="A4:F22"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Registra la equivalencia del Jefe de Produccion (MV y Secado)
'Jefe de Produccion (MV y Secado)' de GE-SO-RL-D35 corresponde al JEFE DE
PRODUCCION del head count, confirmado por Hector: el parentesis precisa las
lineas que el puesto atiende.

Operaciones sube a 19 de 22 cargos (86%) y el total a 56 de 70 (80%), con 81 de
101 personas cubiertas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSq5v2aoJeLSvtorf4qgpi
</commit_message>
<xml_diff>
--- a/Cobertura_IPERC_Administrativos_CAR.xlsx
+++ b/Cobertura_IPERC_Administrativos_CAR.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1. Alcance y criterios'!$A$4:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Resumen por área'!$A$4:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Matriz consolidada'!$A$4:$J$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$H$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5. Observaciones'!$A$4:$G$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$22</definedName>
   </definedNames>
@@ -872,22 +872,22 @@
         <v>22</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>37</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
@@ -1103,22 +1103,22 @@
         <v>70</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>101</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I13" s="14" t="inlineStr"/>
     </row>
@@ -3559,19 +3559,27 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F58" s="17" t="inlineStr">
-        <is>
-          <t>SIN ANALIZAR</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr"/>
-      <c r="H58" s="5" t="inlineStr"/>
+      <c r="F58" s="13" t="inlineStr">
+        <is>
+          <t>ANALIZADO</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>GE-SO-RL-D35</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>Jefe de Producción (MV y Secado)</t>
+        </is>
+      </c>
       <c r="I58" s="9" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>Requiere elaboración de matriz IPERC</t>
+          <t>Denominación distinta entre matriz y head count (equivalencia validada)</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4812,40 +4820,8 @@
       <c r="G18" s="5" t="inlineStr"/>
       <c r="H18" s="5" t="inlineStr"/>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>JEFE DE PRODUCCION</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Quevedo</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>4800 PLANTABAL OPERATIONS MNG STAFF</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Elaborar matriz IPERC para el puesto</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:H19"/>
+  <autoFilter ref="A4:H18"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
@@ -5222,22 +5198,22 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-CC-D1</t>
+          <t>GE-SO-RL-D35</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>QSE &amp; OPERATIONAL EXCELLENCE MANAGER</t>
+          <t>JEFE DE PRODUCCION (MV Y SECADO)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>GERENTE DE CALIDAD Y CERTIFICACIONES</t>
+          <t>JEFE DE PRODUCCION</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>QSE &amp; Operational Excellence</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -5247,7 +5223,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Mismo puesto, distinta denominacion entre matriz y head count</t>
+          <t>Mismo puesto, confirmado por Hector. La matriz precisa entre parentesis las lineas que atiende (MV y Secado)</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -5259,49 +5235,49 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-FI-D1</t>
+          <t>GE-SO-CC-D1</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>JEFE DE CONTABILIDAD E IMPUESTOS</t>
+          <t>QSE &amp; OPERATIONAL EXCELLENCE MANAGER</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>(no consta)</t>
+          <t>GERENTE DE CALIDAD Y CERTIFICACIONES</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>IT&amp;FIN</t>
+          <t>QSE &amp; Operational Excellence</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Cargo nuevo no registrado</t>
+          <t>Equivalencia de denominación</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>ANALIZADO en matriz / NO CONSTA en head count V1.1</t>
+          <t>Mismo puesto, distinta denominacion entre matriz y head count</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Incorporar el cargo a la base de head count</t>
+          <t>Unificar la denominación en la matriz según el head count</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-TH-D1</t>
+          <t>GE-SO-FI-D1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>PEOPLE OPERATIONS PARTNER</t>
+          <t>JEFE DE CONTABILIDAD E IMPUESTOS</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -5311,7 +5287,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>ADM-L&amp;RH</t>
+          <t>IT&amp;FIN</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -5333,66 +5309,70 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-FI-D1</t>
+          <t>GE-SO-TH-D1</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>COORDINADOR DE TESORERIA</t>
+          <t>PEOPLE OPERATIONS PARTNER</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>(no existe)</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr"/>
+          <t>(no consta)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>ADM-L&amp;RH</t>
+        </is>
+      </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Cargo obsoleto</t>
+          <t>Cargo nuevo no registrado</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>CARGO INEXISTENTE - suprimido de la estructura</t>
+          <t>ANALIZADO en matriz / NO CONSTA en head count V1.1</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>ELIMINAR el bloque completo de la matriz GE-SO-FI-D1</t>
+          <t>Incorporar el cargo a la base de head count</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-RL-D35</t>
+          <t>GE-SO-FI-D1</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Jefe de Producción (MV y Secado)</t>
+          <t>COORDINADOR DE TESORERIA</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>(no consta)</t>
+          <t>(no existe)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>SIN CLASIFICAR - detectado este mes</t>
+          <t>Cargo obsoleto</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Puesto evaluado en la matriz que no aparece en el head count del mes</t>
+          <t>CARGO INEXISTENTE - suprimido de la estructura</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Definir si es cargo nuevo, denominación alterna o cargo suprimido</t>
+          <t>ELIMINAR el bloque completo de la matriz GE-SO-FI-D1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Valida los renombres de GE-SO-SF-D1 y admite denominaciones multiples
Una equivalencia puede declarar ahora varias denominaciones del head count para
un mismo puesto evaluado, en lugar de una sola. Asi un renombre no abre una
brecha falsa: el puesto queda cubierto tanto si el head count lo nombra de la
forma anterior como de la nueva, y los cortes de distintos meses se procesan sin
tener que elegir una de las dos.

GE-SO-SF-D1 evalua 'Medico Ocupacional' y 'Auxiliar de servicios de salud', que
el head count de octubre denomina MEDICO y AUXILIAR DE SERVICIOS DE SALUD, y el
V1.1 denominaba MEDICO OCUPACIONAL y AUXILIAR ADMINISTRATIVO. Renombres
confirmados por Hector; ambas denominaciones quedan aceptadas.

El cruce de octubre sube a 56 de 69 cargos (81%). El consolidado sobre el head
count V1.1 se mantiene en 56 de 70 y 81 de 101 personas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSq5v2aoJeLSvtorf4qgpi
</commit_message>
<xml_diff>
--- a/Cobertura_IPERC_Administrativos_CAR.xlsx
+++ b/Cobertura_IPERC_Administrativos_CAR.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Resumen por área'!$A$4:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Matriz consolidada'!$A$4:$J$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$H$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5. Observaciones'!$A$4:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5. Observaciones'!$A$4:$G$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -564,7 +564,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4858,7 +4858,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
         </is>
       </c>
     </row>
@@ -5023,7 +5023,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>AUXILIAR ADMINISTRATIVO</t>
+          <t>AUXILIAR DE SERVICIOS DE SALUD / AUXILIAR ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>En el head count consta como AUXILIAR ADMINISTRATIVO. La denominacion 'Auxiliar de servicios de salud' se uso solo a efectos de la matriz de Salud Ocupacional. Corresponde al auxiliar administrativo asignado a ADM-L&amp;RH (1 persona); los 5 de Operaciones estan cubiertos por GE-SO-MA-D1.</t>
+          <t>El head count de octubre 2026 adopto la denominacion de la matriz; antes constaba como AUXILIAR ADMINISTRATIVO. Se aceptan ambas.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -5235,22 +5235,22 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-CC-D1</t>
+          <t>GE-SO-SF-D1</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>QSE &amp; OPERATIONAL EXCELLENCE MANAGER</t>
+          <t>MEDICO OCUPACIONAL</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>GERENTE DE CALIDAD Y CERTIFICACIONES</t>
+          <t>MEDICO OCUPACIONAL / MEDICO</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>QSE &amp; Operational Excellence</t>
+          <t>ADM-L&amp;RH</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Mismo puesto, distinta denominacion entre matriz y head count</t>
+          <t>El head count de octubre 2026 renombro el cargo de MEDICO OCUPACIONAL a MEDICO. Se aceptan ambas denominaciones.</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -5272,49 +5272,49 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-FI-D1</t>
+          <t>GE-SO-CC-D1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>JEFE DE CONTABILIDAD E IMPUESTOS</t>
+          <t>QSE &amp; OPERATIONAL EXCELLENCE MANAGER</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>(no consta)</t>
+          <t>GERENTE DE CALIDAD Y CERTIFICACIONES</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>IT&amp;FIN</t>
+          <t>QSE &amp; Operational Excellence</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Cargo nuevo no registrado</t>
+          <t>Equivalencia de denominación</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>ANALIZADO en matriz / NO CONSTA en head count V1.1</t>
+          <t>Mismo puesto, distinta denominacion entre matriz y head count</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Incorporar el cargo a la base de head count</t>
+          <t>Unificar la denominación en la matriz según el head count</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-TH-D1</t>
+          <t>GE-SO-FI-D1</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>PEOPLE OPERATIONS PARTNER</t>
+          <t>JEFE DE CONTABILIDAD E IMPUESTOS</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>ADM-L&amp;RH</t>
+          <t>IT&amp;FIN</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -5346,38 +5346,75 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>GE-SO-TH-D1</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>PEOPLE OPERATIONS PARTNER</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>(no consta)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>ADM-L&amp;RH</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Cargo nuevo no registrado</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>ANALIZADO en matriz / NO CONSTA en head count V1.1</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Incorporar el cargo a la base de head count</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>GE-SO-FI-D1</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>COORDINADOR DE TESORERIA</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>(no existe)</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Cargo obsoleto</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>CARGO INEXISTENTE - suprimido de la estructura</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>ELIMINAR el bloque completo de la matriz GE-SO-FI-D1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G17"/>
+  <autoFilter ref="A4:G18"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -5413,7 +5450,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 06/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Incorpora la matriz de Supervisores de Produccion
GE-SO-PD-D2 evalua el Supervisor de produccion con 76 lineas de riesgo, la
matriz mas extensa del catalogo para un unico puesto. Cierra la brecha mas
pesada del control: siete personas, el 37% de todo el personal que quedaba sin
cubrir.

Operaciones sube de 86% a 91% en cargos y de 75% a 94% en personas. El total
pasa a 59 de 71 cargos (83%) y 87 de 99 personas (88%).

Quedan 12 brechas, todas de una sola persona cada una.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSq5v2aoJeLSvtorf4qgpi
</commit_message>
<xml_diff>
--- a/Cobertura_IPERC_Administrativos_CAR.xlsx
+++ b/Cobertura_IPERC_Administrativos_CAR.xlsx
@@ -13,16 +13,14 @@
     <sheet name="4. Brechas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. Observaciones" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Trazabilidad" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7. Cambios del mes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1. Alcance y criterios'!$A$4:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Resumen por área'!$A$4:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Matriz consolidada'!$A$4:$J$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4. Brechas'!$A$4:$H$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5. Observaciones'!$A$4:$G$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'7. Cambios del mes'!$A$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6. Trazabilidad'!$A$4:$F$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +564,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -780,7 +778,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -867,29 +865,29 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Gerencia</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
@@ -900,26 +898,26 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Gerencia</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>2</v>
@@ -1105,22 +1103,22 @@
         <v>71</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>99</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I13" s="14" t="inlineStr"/>
     </row>
@@ -1165,7 +1163,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -3833,21 +3831,25 @@
           <t>Quevedo</t>
         </is>
       </c>
-      <c r="F64" s="17" t="inlineStr">
-        <is>
-          <t>SIN ANALIZAR</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr"/>
-      <c r="H64" s="5" t="inlineStr"/>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>ANALIZADO</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>GE-SO-PD-D2</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor de producción</t>
+        </is>
+      </c>
       <c r="I64" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" s="5" t="inlineStr">
-        <is>
-          <t>Requiere elaboración de matriz IPERC</t>
-        </is>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="J64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4353,7 +4355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4376,7 +4378,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -4425,16 +4427,16 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>ADM-L&amp;RH</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>SUPERVISOR DE PRODUCCIÓN</t>
+          <t>COORDINADOR DE SEGURIDAD FISICA</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -4443,7 +4445,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>3010 KITS PRODUCTION - PGS / 3821 SUP DE PRODUCCION</t>
+          <t>1200 PLANTATION MANAGEMENT</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -4457,12 +4459,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>ADM-L&amp;RH</t>
+          <t>Gerencia</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>COORDINADOR DE SEGURIDAD FISICA</t>
+          <t>CHOFER</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
@@ -4470,12 +4472,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Quevedo</t>
+          <t>Samborondon</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>1200 PLANTATION MANAGEMENT</t>
+          <t>5800 GENERAL MANAGEMENT</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -4494,7 +4496,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>CHOFER</t>
+          <t>GERENTE GENERAL</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -4502,7 +4504,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Samborondon</t>
+          <t>Quevedo</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -4521,12 +4523,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Gerencia</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>GERENTE GENERAL</t>
+          <t>JUNIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
@@ -4534,12 +4536,12 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Quevedo</t>
+          <t>Samborondon</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>5800 GENERAL MANAGEMENT</t>
+          <t>5930 3ACM Expenses</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -4553,12 +4555,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>IT&amp;FIN</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>JUNIOR BUSINESS CONTROLLER</t>
+          <t>ANALISTA DE IMPUESTOS</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
@@ -4571,7 +4573,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>5930 3ACM Expenses</t>
+          <t>5300 FINANCE</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -4590,7 +4592,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>ANALISTA DE IMPUESTOS</t>
+          <t>DIRECTOR FINANCIERO</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
@@ -4622,7 +4624,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>DIRECTOR FINANCIERO</t>
+          <t>GERENTE FINANCIERO</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -4654,7 +4656,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>GERENTE FINANCIERO</t>
+          <t>JEFE  DE DESARROLLO DE APLICACIONES</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
@@ -4667,7 +4669,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>5300 FINANCE</t>
+          <t>5400 IT</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -4686,7 +4688,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>JEFE  DE DESARROLLO DE APLICACIONES</t>
+          <t>JUNIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -4699,7 +4701,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>5400 IT</t>
+          <t>5934 BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -4718,7 +4720,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>JUNIOR BUSINESS CONTROLLER</t>
+          <t>SENIOR BUSINESS CONTROLLER</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
@@ -4745,12 +4747,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>IT&amp;FIN</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>SENIOR BUSINESS CONTROLLER</t>
+          <t>APRENDIZ</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -4758,12 +4760,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Samborondon</t>
+          <t>Quevedo</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>5934 BUSINESS CONTROLLER</t>
+          <t>3801 PLANTABAL MANTENANCE #1</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -4782,7 +4784,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>APRENDIZ</t>
+          <t>JEFE DE BODEGA</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
@@ -4795,7 +4797,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>3801 PLANTABAL MANTENANCE #1</t>
+          <t>2500 SERVICE CENTER</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -4806,40 +4808,8 @@
       <c r="G16" s="5" t="inlineStr"/>
       <c r="H16" s="5" t="inlineStr"/>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>JEFE DE BODEGA</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Quevedo</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>2500 SERVICE CENTER</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Elaborar matriz IPERC para el puesto</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:H17"/>
+  <autoFilter ref="A4:H16"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
@@ -4876,7 +4846,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5505,7 +5475,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
+          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -5824,622 +5794,245 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-PGS-D1</t>
+          <t>GE-SO-PD-D2</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Engicore</t>
+          <t>Supervisor de producción</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Jefe de Diseño e Ingenieria (9) · Ingeniero de Diseño e Ingenieria (14) · Analista de Diseño e Ingenieria (9)</t>
+          <t>Supervisor de producción (76)</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>f4a8175b-GE-SO-PGS-D1_-_Engicore.xlsx</t>
+          <t>92b21579-GE-SO-PD-D2_-_Supervisores_de_Producci_n.xlsx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-PO-D1</t>
+          <t>GE-SO-PGS-D1</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Planificación y Logística</t>
+          <t>Engicore</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Jefe de Planificación y Logística (11) · Coordinador de Supply Chain (6) · Programador de Producción (8) · Analista de Supply Chain (6)</t>
+          <t>Jefe de Diseño e Ingenieria (9) · Ingeniero de Diseño e Ingenieria (14) · Analista de Diseño e Ingenieria (9)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>1fa9982d-GE-SO-PO-D1_-_Planificaci_n_y_Log_stica.xlsx</t>
+          <t>f4a8175b-GE-SO-PGS-D1_-_Engicore.xlsx</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-PY-D1</t>
+          <t>GE-SO-PO-D1</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Proyectos</t>
+          <t>Planificación y Logística</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Jefe de Proyectos (20) · Ingeniero de Proyectos (15) · Analista de Proyectos (16)</t>
+          <t>Jefe de Planificación y Logística (11) · Coordinador de Supply Chain (6) · Programador de Producción (8) · Analista de Supply Chain (6)</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>933cde5a-GE-SO-PY-D1_-_Proyectos.xlsx</t>
+          <t>1fa9982d-GE-SO-PO-D1_-_Planificaci_n_y_Log_stica.xlsx</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-RL-D35</t>
+          <t>GE-SO-PY-D1</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Operations Mng Staff</t>
+          <t>Proyectos</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Director de Operaciones (14) · Gerente de Producción (16) · Jefe de Producción (MV y Secado) (18) · Auxiliar Administrativo (12)</t>
+          <t>Jefe de Proyectos (20) · Ingeniero de Proyectos (15) · Analista de Proyectos (16)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>fe6c6893-Matriz_IPERC_Plantabal_Operations_Mng_Staff.xlsx</t>
+          <t>933cde5a-GE-SO-PY-D1_-_Proyectos.xlsx</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-SC-D1</t>
+          <t>GE-SO-RL-D35</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Operations Mng Staff</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Analista Supply Chain (13) · Analista Compras (14) · Jefe de Compras (13)</t>
+          <t>Director de Operaciones (14) · Gerente de Producción (16) · Jefe de Producción (MV y Secado) (18) · Auxiliar Administrativo (12)</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>9c752964-GE-SO-SC-D1_-_Compras.xlsx</t>
+          <t>fe6c6893-Matriz_IPERC_Plantabal_Operations_Mng_Staff.xlsx</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>GE-SO-SF-D1</t>
+          <t>GE-SO-SC-D1</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Salud Ocupacional</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Medico Ocupacional (18) · Enfermero Ocupacional (10) · Auxiliar de servicios de salud (11)</t>
+          <t>Analista Supply Chain (13) · Analista Compras (14) · Jefe de Compras (13)</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>cf092d8f-GE-SO-SF-D1_-_Salud_ocupacional.xlsx</t>
+          <t>9c752964-GE-SO-SC-D1_-_Compras.xlsx</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>GE-SO-TH-D1</t>
+          <t>GE-SO-SF-D1</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>RECURSOS HUMANOS</t>
+          <t>Salud Ocupacional</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>339</v>
+        <v>39</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>HR DIRECTOR AMERICAS (36) · HR BUSINNES PARTNER AMERICAS (42) · BUSINNES PARTNER DE RECURSOS HUMANOS (28) · COORDINADORA DE DESARROLLO ORGANIZACIONAL (49) · PEOPLE OPERATIONS PARTNER (42) · ANALISTA DE RECURSOS HUMANOS (72) · ANALISTA DE RECURSOS HUMANOS Y NÓMINA (28) · ANALISTA DE DESARROLLO ORGANIZACIONAL (42)</t>
+          <t>Medico Ocupacional (18) · Enfermero Ocupacional (10) · Auxiliar de servicios de salud (11)</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>b206b7b5-GE-SO-TH-D1_-_RRHH.xlsx</t>
+          <t>cf092d8f-GE-SO-SF-D1_-_Salud_ocupacional.xlsx</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>GE-SO-TH-D1</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>RECURSOS HUMANOS</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>339</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>HR DIRECTOR AMERICAS (36) · HR BUSINNES PARTNER AMERICAS (42) · BUSINNES PARTNER DE RECURSOS HUMANOS (28) · COORDINADORA DE DESARROLLO ORGANIZACIONAL (49) · PEOPLE OPERATIONS PARTNER (42) · ANALISTA DE RECURSOS HUMANOS (72) · ANALISTA DE RECURSOS HUMANOS Y NÓMINA (28) · ANALISTA DE DESARROLLO ORGANIZACIONAL (42)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>b206b7b5-GE-SO-TH-D1_-_RRHH.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr"/>
-      <c r="C22" s="9" t="n">
-        <v>59</v>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>1179</v>
-      </c>
-      <c r="E22" s="5" t="inlineStr"/>
-      <c r="F22" s="5" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>1255</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F22"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>CAMBIOS RESPECTO AL CORTE ANTERIOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>PLANTACIONES DE BALSA PLANTABAL S.A. / 3A CORE MATERIALS  ·  Control de cobertura IPERC - Personal administrativo  ·  Corte 14/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tipo de cambio</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Área</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Cargo</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>N° personas</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Estado de cobertura</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Acción sugerida</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>ALTA - cargo nuevo</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>ADM-L&amp;RH</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>AUXILIAR DE SERVICIOS DE SALUD</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Verificar cobertura</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Confirmar si existe matriz IPERC que cubra el puesto</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>ALTA - cargo nuevo</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>ADM-L&amp;RH</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>COORDINADOR DE SEGURIDAD FISICA</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Verificar cobertura</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Confirmar si existe matriz IPERC que cubra el puesto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>ALTA - cargo nuevo</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>ADM-L&amp;RH</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>MEDICO</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Verificar cobertura</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Confirmar si existe matriz IPERC que cubra el puesto</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>ALTA - cargo nuevo</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>ADM-L&amp;RH</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>PEOPLE OPERATIONS PARTNER</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Verificar cobertura</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Confirmar si existe matriz IPERC que cubra el puesto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>VARIACIÓN de dotación (2 → 1)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>IT&amp;FIN</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>COORDINADOR CONTABLE</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Sin acción si el cargo ya está cubierto</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>ALTA - cargo nuevo</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>IT&amp;FIN</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>JEFE DE CONTABILIDAD E IMPUESTOS</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Verificar cobertura</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Confirmar si existe matriz IPERC que cubra el puesto</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>VARIACIÓN de dotación (3 → 2)</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>TECNICO DE INVENTARIO</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Sin acción si el cargo ya está cubierto</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>VARIACIÓN de dotación (4 → 3)</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>QSE &amp; Operational Excellence</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>TECNICO DE CALIDAD</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Sin acción si el cargo ya está cubierto</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>BAJA - cargo ya no consta</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>ADM-L&amp;RH</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>AUXILIAR ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Evaluar si corresponde retirar el bloque de la matriz IPERC</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>BAJA - cargo ya no consta</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>ADM-L&amp;RH</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>MÉDICO OCUPACIONAL</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Evaluar si corresponde retirar el bloque de la matriz IPERC</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>BAJA - cargo ya no consta</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>IT&amp;FIN</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>ANALISTA DE REDES</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Evaluar si corresponde retirar el bloque de la matriz IPERC</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>BAJA - cargo ya no consta</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>IT&amp;FIN</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>MENSAJERO / REPARTIDOR</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5" t="inlineStr"/>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Evaluar si corresponde retirar el bloque de la matriz IPERC</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:F16"/>
+  <autoFilter ref="A4:F23"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>